<commit_message>
updated Framework diagram to include new layers and updated governance framework. Added new diagram to docs folder and updated test results in evidence folder.
</commit_message>
<xml_diff>
--- a/evidence/test-results-final.xlsx
+++ b/evidence/test-results-final.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11835" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11832"/>
   </bookViews>
   <sheets>
     <sheet name="Layer 1 Test Cases" sheetId="1" r:id="rId1"/>
@@ -2311,35 +2311,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="12">
     <dxf>
       <fill>
         <patternFill>
@@ -2421,27 +2393,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2722,20 +2673,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultColWidth="28" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="28" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="63.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="63.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="100" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.109375" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="28" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="6" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2764,7 +2715,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
@@ -2791,7 +2742,7 @@
       </c>
       <c r="I2" s="9"/>
     </row>
-    <row r="3" spans="1:9" ht="255" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
@@ -2817,7 +2768,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
@@ -2843,7 +2794,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="240" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
@@ -2869,7 +2820,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
@@ -2895,7 +2846,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="360" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
@@ -2921,7 +2872,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="315" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>26</v>
       </c>
@@ -2947,7 +2898,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="300" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>28</v>
       </c>
@@ -2973,7 +2924,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="300" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="288" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>30</v>
       </c>
@@ -2999,7 +2950,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
@@ -3025,7 +2976,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>35</v>
       </c>
@@ -3051,7 +3002,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="180" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>37</v>
       </c>
@@ -3077,7 +3028,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="375" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>40</v>
       </c>
@@ -3103,7 +3054,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>42</v>
       </c>
@@ -3129,7 +3080,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>44</v>
       </c>
@@ -3155,7 +3106,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>46</v>
       </c>
@@ -3181,7 +3132,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="330" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>71</v>
       </c>
@@ -3207,77 +3158,77 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D20" s="18" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D21" s="17" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D22" s="18" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="D23" s="19" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D24" s="19" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D25" s="19" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D27" s="16" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="D28" s="7" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D29" s="7" t="s">
         <v>184</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="beginsWith" dxfId="15" priority="5" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="11" priority="5" operator="beginsWith" text="PASS">
       <formula>LEFT(H2,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:I7 B9:C9 A8:A19 D8:I18 B11:C18 B10">
-    <cfRule type="beginsWith" dxfId="14" priority="4" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="10" priority="4" operator="beginsWith" text="FAIL">
       <formula>LEFT(A1,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H18">
-    <cfRule type="beginsWith" dxfId="13" priority="3" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="9" priority="3" operator="beginsWith" text="PASS">
       <formula>LEFT(H4,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="beginsWith" dxfId="12" priority="2" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="8" priority="2" operator="beginsWith" text="FAIL">
       <formula>LEFT(B8,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8">
-    <cfRule type="beginsWith" dxfId="11" priority="1" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="7" priority="1" operator="beginsWith" text="FAIL">
       <formula>LEFT(C8,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3289,20 +3240,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultColWidth="39.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="39.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="86.85546875" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="49.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="86.88671875" customWidth="1"/>
+    <col min="5" max="5" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="49.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3331,7 +3282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>88</v>
       </c>
@@ -3358,7 +3309,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>90</v>
       </c>
@@ -3385,7 +3336,7 @@
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>92</v>
       </c>
@@ -3412,7 +3363,7 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>94</v>
       </c>
@@ -3439,7 +3390,7 @@
       </c>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>96</v>
       </c>
@@ -3466,7 +3417,7 @@
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>98</v>
       </c>
@@ -3493,7 +3444,7 @@
       </c>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>100</v>
       </c>
@@ -3520,7 +3471,7 @@
       </c>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>102</v>
       </c>
@@ -3547,7 +3498,7 @@
       </c>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>104</v>
       </c>
@@ -3574,7 +3525,7 @@
       </c>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>106</v>
       </c>
@@ -3593,17 +3544,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:I1">
-    <cfRule type="beginsWith" dxfId="10" priority="3" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="6" priority="3" operator="beginsWith" text="FAIL">
       <formula>LEFT(A1,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H10">
-    <cfRule type="beginsWith" dxfId="9" priority="2" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="PASS">
       <formula>LEFT(H2,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:H10">
-    <cfRule type="beginsWith" dxfId="8" priority="1" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="4" priority="1" operator="beginsWith" text="FAIL">
       <formula>LEFT(G2,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3615,20 +3566,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultColWidth="52.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="52.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
-    <col min="4" max="4" width="55.5703125" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="55.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="61.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3657,7 +3608,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="180" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>140</v>
       </c>
@@ -3684,7 +3635,7 @@
       </c>
       <c r="I2" s="11"/>
     </row>
-    <row r="3" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>141</v>
       </c>
@@ -3711,7 +3662,7 @@
       </c>
       <c r="I3" s="11"/>
     </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>142</v>
       </c>
@@ -3738,7 +3689,7 @@
       </c>
       <c r="I4" s="11"/>
     </row>
-    <row r="5" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>143</v>
       </c>
@@ -3765,7 +3716,7 @@
       </c>
       <c r="I5" s="11"/>
     </row>
-    <row r="6" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>144</v>
       </c>
@@ -3792,7 +3743,7 @@
       </c>
       <c r="I6" s="11"/>
     </row>
-    <row r="7" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>145</v>
       </c>
@@ -3819,7 +3770,7 @@
       </c>
       <c r="I7" s="11"/>
     </row>
-    <row r="8" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="144" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>146</v>
       </c>
@@ -3846,7 +3797,7 @@
       </c>
       <c r="I8" s="11"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>147</v>
       </c>
@@ -3867,7 +3818,7 @@
       </c>
       <c r="I9" s="11"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>148</v>
       </c>
@@ -3888,27 +3839,27 @@
       </c>
       <c r="I10" s="11"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:I1 G2:H5 G7:H10">
-    <cfRule type="beginsWith" dxfId="7" priority="6" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="3" priority="6" operator="beginsWith" text="FAIL">
       <formula>LEFT(A1,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H5 H7:H10">
-    <cfRule type="beginsWith" dxfId="6" priority="5" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="2" priority="5" operator="beginsWith" text="PASS">
       <formula>LEFT(H2,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:H6">
-    <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="FAIL">
       <formula>LEFT(G6,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6">
-    <cfRule type="beginsWith" dxfId="4" priority="1" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="PASS">
       <formula>LEFT(H6,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
updated customer auto tfvars file to include new plug and play configuration and updated test results in the evidence directory.
</commit_message>
<xml_diff>
--- a/evidence/test-results-final.xlsx
+++ b/evidence/test-results-final.xlsx
@@ -2311,7 +2311,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="14">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3208,28 +3222,33 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H2:H3">
-    <cfRule type="beginsWith" dxfId="11" priority="5" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="13" priority="6" operator="beginsWith" text="PASS">
       <formula>LEFT(H2,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:I7 B9:C9 A8:A19 D8:I18 B11:C18 B10">
-    <cfRule type="beginsWith" dxfId="10" priority="4" operator="beginsWith" text="FAIL">
+  <conditionalFormatting sqref="A1:I1 B9:C9 A8:A19 D8:I18 B11:C18 B10 A3:I7 B2:I2">
+    <cfRule type="beginsWith" dxfId="12" priority="5" operator="beginsWith" text="FAIL">
       <formula>LEFT(A1,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H18">
-    <cfRule type="beginsWith" dxfId="9" priority="3" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="11" priority="4" operator="beginsWith" text="PASS">
       <formula>LEFT(H4,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="beginsWith" dxfId="8" priority="2" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="10" priority="3" operator="beginsWith" text="FAIL">
       <formula>LEFT(B8,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8">
-    <cfRule type="beginsWith" dxfId="7" priority="1" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="9" priority="2" operator="beginsWith" text="FAIL">
       <formula>LEFT(C8,LEN("FAIL"))="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="beginsWith" dxfId="1" priority="1" operator="beginsWith" text="FAIL">
+      <formula>LEFT(A2,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3544,17 +3563,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:I1">
-    <cfRule type="beginsWith" dxfId="6" priority="3" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="8" priority="3" operator="beginsWith" text="FAIL">
       <formula>LEFT(A1,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H10">
-    <cfRule type="beginsWith" dxfId="5" priority="2" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="7" priority="2" operator="beginsWith" text="PASS">
       <formula>LEFT(H2,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:H10">
-    <cfRule type="beginsWith" dxfId="4" priority="1" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="6" priority="1" operator="beginsWith" text="FAIL">
       <formula>LEFT(G2,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3844,22 +3863,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:I1 G2:H5 G7:H10">
-    <cfRule type="beginsWith" dxfId="3" priority="6" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="5" priority="6" operator="beginsWith" text="FAIL">
       <formula>LEFT(A1,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H5 H7:H10">
-    <cfRule type="beginsWith" dxfId="2" priority="5" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="4" priority="5" operator="beginsWith" text="PASS">
       <formula>LEFT(H2,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:H6">
-    <cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="FAIL">
+    <cfRule type="beginsWith" dxfId="3" priority="2" operator="beginsWith" text="FAIL">
       <formula>LEFT(G6,LEN("FAIL"))="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6">
-    <cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="PASS">
+    <cfRule type="beginsWith" dxfId="2" priority="1" operator="beginsWith" text="PASS">
       <formula>LEFT(H6,LEN("PASS"))="PASS"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>